<commit_message>
fix: resolve openpyxl merged cells deletion bug that cleared parts 5 and 6 in Excel output
</commit_message>
<xml_diff>
--- a/form_enriched.xlsx
+++ b/form_enriched.xlsx
@@ -12667,19 +12667,8 @@
     <row r="420" ht="25.5" customHeight="1" s="37"/>
     <row r="423" ht="45" customHeight="1" s="37"/>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="B414:E414"/>
-    <mergeCell ref="B420:F420"/>
-    <mergeCell ref="A8:G8"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="B423:F423"/>
-    <mergeCell ref="B418:F418"/>
-    <mergeCell ref="B419:F419"/>
-    <mergeCell ref="E4:G4"/>
-    <mergeCell ref="A7:G7"/>
-    <mergeCell ref="E3:G3"/>
-    <mergeCell ref="B417:F417"/>
+  <mergeCells count="1">
+    <mergeCell ref="B404:E404"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" display="https://www.autoopt.ru/catalog/021853-klapan_zil_kamaz_maz_dvuhprovodnyj_upravlenija_tormozami_pricepa_s_klapanom_obryva_belomo" r:id="rId1"/>

</xml_diff>

<commit_message>
fix: remove part 401 'Текущий ремонт' to make catalog exactly 400 parts
</commit_message>
<xml_diff>
--- a/form_enriched.xlsx
+++ b/form_enriched.xlsx
@@ -681,7 +681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H404"/>
+  <dimension ref="A1:H403"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15.75"/>
   <cols>
     <col width="5.28515625" customWidth="1" style="1" min="1" max="1"/>
@@ -12618,42 +12618,20 @@
       <c r="H402" s="13" t="n"/>
     </row>
     <row r="403">
-      <c r="A403" s="9" t="n"/>
-      <c r="B403" s="19" t="n">
-        <v>401</v>
-      </c>
-      <c r="C403" s="20" t="inlineStr">
-        <is>
-          <t>Текущий ремонт</t>
-        </is>
-      </c>
-      <c r="D403" s="18" t="n"/>
-      <c r="E403" s="39" t="inlineStr">
-        <is>
-          <t>нормо-час</t>
-        </is>
-      </c>
-      <c r="F403" s="12" t="n"/>
-      <c r="G403" t="inlineStr">
-        <is>
-          <t>https://www.autoopt.ru/search/index?search=</t>
-        </is>
-      </c>
-    </row>
-    <row r="404" ht="31.5" customHeight="1" s="37">
-      <c r="B404" s="34" t="inlineStr">
+      <c r="B403" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">ИТОГО С НДС </t>
         </is>
       </c>
-      <c r="C404" s="40" t="n"/>
-      <c r="D404" s="40" t="n"/>
-      <c r="E404" s="41" t="n"/>
-      <c r="F404" s="12">
-        <f>SUM(F3:F403)</f>
+      <c r="C403" s="40" t="n"/>
+      <c r="D403" s="40" t="n"/>
+      <c r="E403" s="41" t="n"/>
+      <c r="F403" s="12">
+        <f>SUM(F3:F402)</f>
         <v/>
       </c>
     </row>
+    <row r="404" ht="31.5" customHeight="1" s="37"/>
     <row r="405" ht="31.5" customHeight="1" s="37"/>
     <row r="406" ht="47.25" customHeight="1" s="37"/>
     <row r="407" ht="31.5" customHeight="1" s="37"/>
@@ -12668,7 +12646,7 @@
     <row r="423" ht="45" customHeight="1" s="37"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B404:E404"/>
+    <mergeCell ref="B403:E403"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" display="https://www.autoopt.ru/catalog/021853-klapan_zil_kamaz_maz_dvuhprovodnyj_upravlenija_tormozami_pricepa_s_klapanom_obryva_belomo" r:id="rId1"/>

</xml_diff>